<commit_message>
added logo and favicon
</commit_message>
<xml_diff>
--- a/scripts/data/publications.xlsx
+++ b/scripts/data/publications.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kamilakolpashnikova/Dropbox/Mac/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34C2746F-C844-ED4F-B4F2-56678D310D8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69E1D1F0-F2C6-964D-A3AB-C35C53BF2DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1880" windowWidth="28040" windowHeight="17180" xr2:uid="{1AE54D6A-986F-F746-921F-6A2F1439D6A6}"/>
+    <workbookView xWindow="44000" yWindow="1140" windowWidth="28040" windowHeight="17180" xr2:uid="{1AE54D6A-986F-F746-921F-6A2F1439D6A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="521">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="629">
   <si>
     <t>Evolution of Semantic Similarity—A Survey</t>
   </si>
@@ -1658,12 +1657,347 @@
   <si>
     <t>International Conference on Frontiers of Intelligent Computing: Theory and …</t>
   </si>
+  <si>
+    <t>Smart fog: Fog computing framework for unsupervised clustering analytics in wearable internet of things</t>
+  </si>
+  <si>
+    <t>D Borthakur, H Dubey, N Constant, L Mahler, K Mankodiya</t>
+  </si>
+  <si>
+    <t>2017 IEEE Global Conference on Signal and Information Processing (GlobalSIP …</t>
+  </si>
+  <si>
+    <t>Fog computing in medical internet-of-things: architecture, implementation, and applications</t>
+  </si>
+  <si>
+    <t>H Dubey, A Monteiro, N Constant, M Abtahi, D Borthakur, L Mahler, Y Sun, ...</t>
+  </si>
+  <si>
+    <t>Handbook of large-scale distributed computing in smart healthcare, 281-321</t>
+  </si>
+  <si>
+    <t>Fog-assisted wiot: A smart fog gateway for end-to-end analytics in wearable internet of things</t>
+  </si>
+  <si>
+    <t>N Constant, D Borthakur, M Abtahi, H Dubey, K Mankodiya</t>
+  </si>
+  <si>
+    <t>arXiv preprint arXiv:1701.08680</t>
+  </si>
+  <si>
+    <t>Fog assisted cloud computing in era of big data and internet-of-things: systems, architectures, and applications</t>
+  </si>
+  <si>
+    <t>RK Barik, H Dubey, C Misra, D Borthakur, N Constant, SA Sasane, ...</t>
+  </si>
+  <si>
+    <t>Cloud computing for optimization: foundations, applications, and challenges …</t>
+  </si>
+  <si>
+    <t>Yoga pose estimation using angle-based feature extraction</t>
+  </si>
+  <si>
+    <t>D Borthakur, A Paul, D Kapil, MJ Saikia</t>
+  </si>
+  <si>
+    <t>Healthcare 11 (24), 3133</t>
+  </si>
+  <si>
+    <t>Associations between police lethal force errors, measures of diurnal and reactive cortisol, and mental health</t>
+  </si>
+  <si>
+    <t>JF Chan, PM Di Nota, K Planche, D Borthakur, JP Andersen</t>
+  </si>
+  <si>
+    <t>Psychoneuroendocrinology 142, 105789</t>
+  </si>
+  <si>
+    <t>SmartEAR: Smartwatch-based unsupervised learning for multi-modal signal analysis in opportunistic sensing framework</t>
+  </si>
+  <si>
+    <t>D Borthakur, A Peltier, H Dubey, JV Gyllinsky, K Mankodiya</t>
+  </si>
+  <si>
+    <t>Proceedings of the 2018 IEEE/ACM International Conference on Connected …</t>
+  </si>
+  <si>
+    <t>Using breath-like cues for guided breathing</t>
+  </si>
+  <si>
+    <t>G Marentakis, D Borthakur, P Batchelor, JP Andersen, V Grace</t>
+  </si>
+  <si>
+    <t>Extended Abstracts of the 2021 CHI Conference on Human Factors in Computing …</t>
+  </si>
+  <si>
+    <t>A machine learning approach to classify working memory load from optical neuroimaging data</t>
+  </si>
+  <si>
+    <t>MJ Saikia, S Kuanar, D Borthakur, M Vinti, T Tendhar</t>
+  </si>
+  <si>
+    <t>Optical Techniques in Neurosurgery, Neurophotonics, and Optogenetics 11629 …</t>
+  </si>
+  <si>
+    <t>Fuzzy C-means clustering and sonification of HRV features</t>
+  </si>
+  <si>
+    <t>D Borthakur, V Grace, P Batchelor, H Dubey, K Mankodiya</t>
+  </si>
+  <si>
+    <t>2019 IEEE/ACM International Conference on Connected Health: Applications …</t>
+  </si>
+  <si>
+    <t>Inequity aversion toward AI counterparts</t>
+  </si>
+  <si>
+    <t>D Borthakur, P Diep, JE Plaks</t>
+  </si>
+  <si>
+    <t>Scientific Reports 15 (1), 37916</t>
+  </si>
+  <si>
+    <t>Machine learning approach for music familiarity classification with single-channel eeg</t>
+  </si>
+  <si>
+    <t>N Kim, D Borthakur, MJ Saikia</t>
+  </si>
+  <si>
+    <t>2024 46th Annual International Conference of the IEEE Engineering in …</t>
+  </si>
+  <si>
+    <t>Empowering bystanders: a psychological and institutional model for intervention in academic bullying</t>
+  </si>
+  <si>
+    <t>D Borthakur, L Crockett, J Mihalchan, J Swann, MJ Saikia</t>
+  </si>
+  <si>
+    <t>Frontiers in Psychology 16, 1650438</t>
+  </si>
+  <si>
+    <t>Cardiorespiratory optimized guided-breathing for post-stress recovery in a group setting</t>
+  </si>
+  <si>
+    <t>D Borthakur</t>
+  </si>
+  <si>
+    <t>Quantifying the Effects of Motor Tasks on Corticokinematic Coherence in Parkinson's Disease</t>
+  </si>
+  <si>
+    <t>University of Rhode Island</t>
+  </si>
+  <si>
+    <t>Artificial Intelligence (AI) in Patient–Healthcare Relationships: Psychosocial Perspective</t>
+  </si>
+  <si>
+    <t>MJ Saikia, D Borthakur</t>
+  </si>
+  <si>
+    <t>IEEE Access</t>
+  </si>
+  <si>
+    <t>Personality Influences on Inequity Aversion Toward Human and AI Counterparts</t>
+  </si>
+  <si>
+    <t>D Borthakur, H Ahmad, JE Plaks</t>
+  </si>
+  <si>
+    <t>Identifying Proposers’ Behavioral Patterns in Human-AI Economic Interactions</t>
+  </si>
+  <si>
+    <t>2025 IEEE International Conference on Future Machine Learning and Data …</t>
+  </si>
+  <si>
+    <t>Assamese Society Through the Lens of Cultural Neuroscience</t>
+  </si>
+  <si>
+    <t>ALOK https://www.alokassamesejournal.com/current-issue 16 (16), 82-88</t>
+  </si>
+  <si>
+    <t>“Prosodic Finder” – A web application</t>
+  </si>
+  <si>
+    <t>DBS Mahanta</t>
+  </si>
+  <si>
+    <t>Conference: 37th International Conference of Linguistics Society of India …</t>
+  </si>
+  <si>
+    <t>Automating Detection of Drug-Related Harms on Social Media: Machine Learning Framework</t>
+  </si>
+  <si>
+    <t>Journal of Medical Internet Research 25, e43630</t>
+  </si>
+  <si>
+    <t>Comparison of Moderated and Unmoderated Remote Usability Sessions for Web-Based Simulation Software: A Randomized Controlled Trial</t>
+  </si>
+  <si>
+    <t>Simulating the Evolution of Homeless Populations in Canada Using Modified Deep Q-Learning (MDQL) and Modified Neural Fitted Q-Iteration (MNFQ) Algorithms</t>
+  </si>
+  <si>
+    <t>Green Communication Protocol with Geolocation</t>
+  </si>
+  <si>
+    <t>G Srivastava, A Fisher, R Bryce, J Crichigno</t>
+  </si>
+  <si>
+    <t>2019 IEEE 89th Vehicular Technology Conference (VTC2019-Spring), 1-6</t>
+  </si>
+  <si>
+    <r>
+      <t>15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="24"/>
+        <color rgb="FF660099"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>*</t>
+    </r>
+  </si>
+  <si>
+    <t>Predicting the Resource Needs and Outcomes of Computationally Intensive Biological Simulations</t>
+  </si>
+  <si>
+    <t>2020 Spring Simulation Conference (SpringSim), 1-12</t>
+  </si>
+  <si>
+    <t>TentNet: Deep Learning Tent Detection Algorithm Using A Synthetic Training Approach</t>
+  </si>
+  <si>
+    <t>Investigating the Implications of COVID-19 for the Rural and Remote Population of Northern Ontario Using a Mathematical Model</t>
+  </si>
+  <si>
+    <t>BEAUT: An ExplainaBle Deep LEarning Model for Agent-Based PopUlations With Poor DaTa</t>
+  </si>
+  <si>
+    <t>PLOS ONE 19 (6), e0303646</t>
+  </si>
+  <si>
+    <t>How Many Costly Simulations Do we Need to Create Accurate Metamodels? A Case Study on Predicting HIV Viral Load in Response to Clinically Relevant Intervention Scenarios</t>
+  </si>
+  <si>
+    <t>International Workshop on Health Intelligence, 273-288</t>
+  </si>
+  <si>
+    <t>HEAL-Summ: A Lightweight and Ethical Framework for Accessible Summarization of Health Information</t>
+  </si>
+  <si>
+    <t>MQTTg: An Android Implementation</t>
+  </si>
+  <si>
+    <t>A Fisher, G Srivastava, R Bryce</t>
+  </si>
+  <si>
+    <t>2019 42nd International Conference on Telecommunications and Signal …</t>
+  </si>
+  <si>
+    <t>Facilitating Learning Outcome Assessment- Development of New Datasets and Analysis of Pre-Trained Language Models</t>
+  </si>
+  <si>
+    <t>An Ethical Visualization of the NorthCOVID-19 Model</t>
+  </si>
+  <si>
+    <t>Development of Simulation and Machine Learning Solutions for Social Issues</t>
+  </si>
+  <si>
+    <t>A Fisher</t>
+  </si>
+  <si>
+    <t>Proportion of Preterm birth and associated factors among mothers who gave birth in Debretabor town health institutions, northwest, Ethiopia</t>
+  </si>
+  <si>
+    <t>DG Mekonen, AE Yismaw, TS Nigussie, WM Ambaw</t>
+  </si>
+  <si>
+    <t>BMC research notes 12 (1), 2</t>
+  </si>
+  <si>
+    <t>Prevalence of post partum modern family planning utilization and associated factors among postpartum mothers in Debre Tabor town, North West Ethiopia, 2018</t>
+  </si>
+  <si>
+    <t>EB Taye, DG Mekonen, TZ Debele</t>
+  </si>
+  <si>
+    <t>BMC research notes 12 (1), 430</t>
+  </si>
+  <si>
+    <t>Repeat induced abortion and associated factors among women seeking abortion care services at Debre Markos town health institutions, Amhara regional state, Ethiopia, 2017</t>
+  </si>
+  <si>
+    <t>MI Waktola, DG Mekonen, TS Nigussie, EA Cherkose, AT Abate</t>
+  </si>
+  <si>
+    <t>BMC research notes 13 (1), 44</t>
+  </si>
+  <si>
+    <t>“I became a person again”: Social inclusion and participation experiences of Ethiopian women post-obstetric fistula surgical repair</t>
+  </si>
+  <si>
+    <t>TZ Debele, D Macdonald, HM Aldersey, Z Mengistu, DG Mekonnen, ...</t>
+  </si>
+  <si>
+    <t>Plos one 19 (7), e0307021</t>
+  </si>
+  <si>
+    <t>Predictors of competency on delivery care service among final year undergraduate midwifery students in higher education institutions of Ethiopia, 2019: A cross sectional study</t>
+  </si>
+  <si>
+    <t>DN Gessesse, BW Yirdaw, DG Mekonen</t>
+  </si>
+  <si>
+    <t>Clinical Epidemiology and Global Health 11, 100730</t>
+  </si>
+  <si>
+    <t>Supporting women after obstetric fistula surgery to enhance their social participation and inclusion</t>
+  </si>
+  <si>
+    <t>T Debele, HM Aldersey, D Macdonald, Z Mengistu, DG Mekonnen, ...</t>
+  </si>
+  <si>
+    <t>International journal of environmental research and public health 21 (9), 1201</t>
+  </si>
+  <si>
+    <t>“It is challenging to face the judgmental gazes”: women with physical disability and perinatal care-seeking in rural Ethiopia: a qualitative case study</t>
+  </si>
+  <si>
+    <t>DG Mekonen, E Snelgrove-Clarke, C Donnelly, EH Engeda, T Debele, ...</t>
+  </si>
+  <si>
+    <t>Disability and Rehabilitation, 1-17</t>
+  </si>
+  <si>
+    <t>Perinatal care experiences of women living with disability in Africa: a qualitative systematic review protocol</t>
+  </si>
+  <si>
+    <t>DG Mekonen, E Snelgrove-Clarke, D Macdonald, C Donnelly, E Engeda</t>
+  </si>
+  <si>
+    <t>JBI Evidence Synthesis 23 (4), 772-780</t>
+  </si>
+  <si>
+    <t>Knowledge of Postpartum Women About Modern Contraceptive Methods and Attitudes Towards its Utilization in Debre Tabor Town, Northwest Ethiopia: A Community-Based Cross …</t>
+  </si>
+  <si>
+    <t>EB Taye, DG Mekonnen, TZ Debele</t>
+  </si>
+  <si>
+    <t>Ethiopian Journal of Health and Biomedical Sciences 13 (1), 57-69</t>
+  </si>
+  <si>
+    <t>Proportion of preterm birth and associated factors among mothers who gave birth in Debretabor town health institutions, northwest, Ethiopia.</t>
+  </si>
+  <si>
+    <t>DGM Dawit Gebeyehu Mekonen, AEY Ayenew Engida Yismaw, ...</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1703,6 +2037,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1725,13 +2065,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2067,7 +2408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63F586DF-5126-0C41-93C9-DC8AF5D22C1E}">
-  <dimension ref="A1:C560"/>
+  <dimension ref="A1:C709"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="86.83203125" customWidth="1"/>
@@ -6685,18 +7026,1683 @@
       <c r="B560" s="3"/>
       <c r="C560" s="4"/>
     </row>
+    <row r="561" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A561" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="B561" s="3">
+        <v>133</v>
+      </c>
+      <c r="C561" s="4">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="562" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A562" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="B562" s="3"/>
+      <c r="C562" s="4"/>
+    </row>
+    <row r="563" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A563" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="B563" s="3"/>
+      <c r="C563" s="4"/>
+    </row>
+    <row r="564" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A564" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="B564" s="3">
+        <v>132</v>
+      </c>
+      <c r="C564" s="4">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="565" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A565" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B565" s="3"/>
+      <c r="C565" s="4"/>
+    </row>
+    <row r="566" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A566" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="B566" s="3"/>
+      <c r="C566" s="4"/>
+    </row>
+    <row r="567" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A567" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="B567" s="3">
+        <v>102</v>
+      </c>
+      <c r="C567" s="4">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="568" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A568" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="B568" s="3"/>
+      <c r="C568" s="4"/>
+    </row>
+    <row r="569" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A569" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="B569" s="3"/>
+      <c r="C569" s="4"/>
+    </row>
+    <row r="570" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A570" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="B570" s="3">
+        <v>89</v>
+      </c>
+      <c r="C570" s="4">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="571" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A571" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="B571" s="3"/>
+      <c r="C571" s="4"/>
+    </row>
+    <row r="572" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A572" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="B572" s="3"/>
+      <c r="C572" s="4"/>
+    </row>
+    <row r="573" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A573" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="B573" s="3">
+        <v>40</v>
+      </c>
+      <c r="C573" s="4">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="574" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A574" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B574" s="3"/>
+      <c r="C574" s="4"/>
+    </row>
+    <row r="575" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A575" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="B575" s="3"/>
+      <c r="C575" s="4"/>
+    </row>
+    <row r="576" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A576" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="B576" s="3">
+        <v>17</v>
+      </c>
+      <c r="C576" s="4">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="577" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A577" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="B577" s="3"/>
+      <c r="C577" s="4"/>
+    </row>
+    <row r="578" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A578" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="B578" s="3"/>
+      <c r="C578" s="4"/>
+    </row>
+    <row r="579" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A579" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="B579" s="3">
+        <v>13</v>
+      </c>
+      <c r="C579" s="4">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="580" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A580" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="B580" s="3"/>
+      <c r="C580" s="4"/>
+    </row>
+    <row r="581" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A581" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B581" s="3"/>
+      <c r="C581" s="4"/>
+    </row>
+    <row r="582" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A582" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="B582" s="3">
+        <v>12</v>
+      </c>
+      <c r="C582" s="4">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="583" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A583" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="B583" s="3"/>
+      <c r="C583" s="4"/>
+    </row>
+    <row r="584" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A584" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="B584" s="3"/>
+      <c r="C584" s="4"/>
+    </row>
+    <row r="585" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A585" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="B585" s="3">
+        <v>11</v>
+      </c>
+      <c r="C585" s="4">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="586" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A586" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="B586" s="3"/>
+      <c r="C586" s="4"/>
+    </row>
+    <row r="587" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A587" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="B587" s="3"/>
+      <c r="C587" s="4"/>
+    </row>
+    <row r="588" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A588" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="B588" s="3">
+        <v>7</v>
+      </c>
+      <c r="C588" s="4">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="589" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A589" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="B589" s="3"/>
+      <c r="C589" s="4"/>
+    </row>
+    <row r="590" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A590" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="B590" s="3"/>
+      <c r="C590" s="4"/>
+    </row>
+    <row r="591" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A591" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="B591" s="3">
+        <v>6</v>
+      </c>
+      <c r="C591" s="4">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="592" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A592" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="B592" s="3"/>
+      <c r="C592" s="4"/>
+    </row>
+    <row r="593" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A593" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="B593" s="3"/>
+      <c r="C593" s="4"/>
+    </row>
+    <row r="594" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A594" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="B594" s="3">
+        <v>5</v>
+      </c>
+      <c r="C594" s="4">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="595" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A595" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="B595" s="3"/>
+      <c r="C595" s="4"/>
+    </row>
+    <row r="596" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A596" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="B596" s="3"/>
+      <c r="C596" s="4"/>
+    </row>
+    <row r="597" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A597" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="B597" s="3">
+        <v>4</v>
+      </c>
+      <c r="C597" s="4">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="598" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A598" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="B598" s="3"/>
+      <c r="C598" s="4"/>
+    </row>
+    <row r="599" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A599" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="B599" s="3"/>
+      <c r="C599" s="4"/>
+    </row>
+    <row r="600" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A600" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="B600" s="3">
+        <v>2</v>
+      </c>
+      <c r="C600" s="4">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="601" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A601" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="B601" s="3"/>
+      <c r="C601" s="4"/>
+    </row>
+    <row r="602" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A602" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="B602" s="3">
+        <v>2</v>
+      </c>
+      <c r="C602" s="4">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="603" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A603" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="B603" s="3"/>
+      <c r="C603" s="4"/>
+    </row>
+    <row r="604" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A604" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B604" s="3"/>
+      <c r="C604" s="4"/>
+    </row>
+    <row r="605" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A605" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="B605" s="3">
+        <v>1</v>
+      </c>
+      <c r="C605" s="4">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="606" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A606" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B606" s="3"/>
+      <c r="C606" s="4"/>
+    </row>
+    <row r="607" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A607" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="B607" s="3"/>
+      <c r="C607" s="4"/>
+    </row>
+    <row r="608" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A608" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="B608" s="3"/>
+      <c r="C608" s="4">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="609" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A609" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="B609" s="3"/>
+      <c r="C609" s="4"/>
+    </row>
+    <row r="610" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A610" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="B610" s="3"/>
+      <c r="C610" s="4">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="611" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A611" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="B611" s="3"/>
+      <c r="C611" s="4"/>
+    </row>
+    <row r="612" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A612" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B612" s="3"/>
+      <c r="C612" s="4"/>
+    </row>
+    <row r="613" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A613" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="B613" s="3"/>
+      <c r="C613" s="4">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="614" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A614" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="B614" s="3"/>
+      <c r="C614" s="4"/>
+    </row>
+    <row r="615" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A615" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="B615" s="3"/>
+      <c r="C615" s="4"/>
+    </row>
+    <row r="616" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A616" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="B616" s="3"/>
+      <c r="C616" s="4">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="617" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A617" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="B617" s="3"/>
+      <c r="C617" s="4"/>
+    </row>
+    <row r="618" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A618" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="B618" s="3"/>
+      <c r="C618" s="4"/>
+    </row>
+    <row r="619" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A619" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="B619" s="3">
+        <v>23</v>
+      </c>
+      <c r="C619" s="6">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="620" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A620" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B620" s="3"/>
+      <c r="C620" s="6"/>
+    </row>
+    <row r="621" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A621" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="B621" s="3"/>
+      <c r="C621" s="6"/>
+    </row>
+    <row r="622" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A622" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="B622" s="3">
+        <v>18</v>
+      </c>
+      <c r="C622" s="6">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="623" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A623" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B623" s="3"/>
+      <c r="C623" s="6"/>
+    </row>
+    <row r="624" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A624" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B624" s="3"/>
+      <c r="C624" s="6"/>
+    </row>
+    <row r="625" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A625" s="1" t="s">
+        <v>579</v>
+      </c>
+      <c r="B625" s="3">
+        <v>18</v>
+      </c>
+      <c r="C625" s="6">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="626" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A626" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B626" s="3"/>
+      <c r="C626" s="6"/>
+    </row>
+    <row r="627" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A627" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B627" s="3"/>
+      <c r="C627" s="6"/>
+    </row>
+    <row r="628" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A628" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="B628" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="C628" s="6">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="629" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A629" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="B629" s="5"/>
+      <c r="C629" s="6"/>
+    </row>
+    <row r="630" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A630" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="B630" s="5"/>
+      <c r="C630" s="6"/>
+    </row>
+    <row r="631" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A631" s="1" t="s">
+        <v>584</v>
+      </c>
+      <c r="B631" s="3">
+        <v>14</v>
+      </c>
+      <c r="C631" s="6">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="632" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A632" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B632" s="3"/>
+      <c r="C632" s="6"/>
+    </row>
+    <row r="633" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A633" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="B633" s="3"/>
+      <c r="C633" s="6"/>
+    </row>
+    <row r="634" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A634" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="B634" s="3">
+        <v>12</v>
+      </c>
+      <c r="C634" s="6">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="635" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A635" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B635" s="3"/>
+      <c r="C635" s="6"/>
+    </row>
+    <row r="636" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A636" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B636" s="3"/>
+      <c r="C636" s="6"/>
+    </row>
+    <row r="637" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A637" s="1" t="s">
+        <v>587</v>
+      </c>
+      <c r="B637" s="3">
+        <v>9</v>
+      </c>
+      <c r="C637" s="6">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="638" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A638" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B638" s="3"/>
+      <c r="C638" s="6"/>
+    </row>
+    <row r="639" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A639" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B639" s="3"/>
+      <c r="C639" s="6"/>
+    </row>
+    <row r="640" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A640" s="1" t="s">
+        <v>588</v>
+      </c>
+      <c r="B640" s="3">
+        <v>7</v>
+      </c>
+      <c r="C640" s="6">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="641" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A641" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B641" s="3"/>
+      <c r="C641" s="6"/>
+    </row>
+    <row r="642" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A642" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B642" s="3"/>
+      <c r="C642" s="6"/>
+    </row>
+    <row r="643" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A643" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B643" s="3">
+        <v>6</v>
+      </c>
+      <c r="C643" s="6">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="644" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A644" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B644" s="3"/>
+      <c r="C644" s="6"/>
+    </row>
+    <row r="645" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A645" s="2" t="s">
+        <v>589</v>
+      </c>
+      <c r="B645" s="3"/>
+      <c r="C645" s="6"/>
+    </row>
+    <row r="646" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A646" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="B646" s="3">
+        <v>5</v>
+      </c>
+      <c r="C646" s="6">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="647" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A647" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B647" s="3"/>
+      <c r="C647" s="6"/>
+    </row>
+    <row r="648" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A648" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B648" s="3"/>
+      <c r="C648" s="6"/>
+    </row>
+    <row r="649" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A649" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B649" s="3">
+        <v>3</v>
+      </c>
+      <c r="C649" s="6">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="650" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A650" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B650" s="3"/>
+      <c r="C650" s="6"/>
+    </row>
+    <row r="651" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A651" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="B651" s="3"/>
+      <c r="C651" s="6"/>
+    </row>
+    <row r="652" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A652" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="B652" s="3">
+        <v>2</v>
+      </c>
+      <c r="C652" s="6">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="653" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A653" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B653" s="3"/>
+      <c r="C653" s="6"/>
+    </row>
+    <row r="654" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A654" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="B654" s="3"/>
+      <c r="C654" s="6"/>
+    </row>
+    <row r="655" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A655" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="B655" s="3">
+        <v>2</v>
+      </c>
+      <c r="C655" s="6">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="656" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A656" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="B656" s="3"/>
+      <c r="C656" s="6"/>
+    </row>
+    <row r="657" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A657" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B657" s="3"/>
+      <c r="C657" s="6"/>
+    </row>
+    <row r="658" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A658" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="B658" s="3">
+        <v>1</v>
+      </c>
+      <c r="C658" s="6">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="659" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A659" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="B659" s="3"/>
+      <c r="C659" s="6"/>
+    </row>
+    <row r="660" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A660" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="B660" s="3"/>
+      <c r="C660" s="6"/>
+    </row>
+    <row r="661" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A661" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="B661" s="3">
+        <v>1</v>
+      </c>
+      <c r="C661" s="6">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="662" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A662" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="B662" s="3"/>
+      <c r="C662" s="6"/>
+    </row>
+    <row r="663" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A663" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="B663" s="3"/>
+      <c r="C663" s="6"/>
+    </row>
+    <row r="664" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A664" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="B664" s="3"/>
+      <c r="C664" s="6">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="665" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A665" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="B665" s="3"/>
+      <c r="C665" s="6"/>
+    </row>
+    <row r="666" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A666" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="B666" s="3"/>
+      <c r="C666" s="6"/>
+    </row>
+    <row r="667" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A667" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="B667" s="3"/>
+      <c r="C667" s="6">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="668" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A668" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="B668" s="3"/>
+      <c r="C668" s="6"/>
+    </row>
+    <row r="669" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A669" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="B669" s="3"/>
+      <c r="C669" s="6"/>
+    </row>
+    <row r="670" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A670" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="B670" s="3"/>
+      <c r="C670" s="6">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="671" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A671" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="B671" s="3"/>
+      <c r="C671" s="6"/>
+    </row>
+    <row r="672" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A672" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="B672" s="3"/>
+      <c r="C672" s="6"/>
+    </row>
+    <row r="673" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A673" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="B673" s="3"/>
+      <c r="C673" s="6">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="674" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A674" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="B674" s="3"/>
+      <c r="C674" s="6"/>
+    </row>
+    <row r="675" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A675" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="B675" s="3"/>
+      <c r="C675" s="6"/>
+    </row>
+    <row r="676" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A676" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="B676" s="3"/>
+      <c r="C676" s="6">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="677" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A677" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="B677" s="3"/>
+      <c r="C677" s="6"/>
+    </row>
+    <row r="678" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A678" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="B678" s="3"/>
+      <c r="C678" s="6"/>
+    </row>
+    <row r="679" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A679" s="1" t="s">
+        <v>598</v>
+      </c>
+      <c r="B679" s="3"/>
+      <c r="C679" s="6">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="680" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A680" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="B680" s="3"/>
+      <c r="C680" s="6"/>
+    </row>
+    <row r="681" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A681" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="B681" s="3">
+        <v>59</v>
+      </c>
+      <c r="C681" s="4">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="682" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A682" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="B682" s="3"/>
+      <c r="C682" s="4"/>
+    </row>
+    <row r="683" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A683" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="B683" s="3"/>
+      <c r="C683" s="4"/>
+    </row>
+    <row r="684" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A684" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="B684" s="3">
+        <v>42</v>
+      </c>
+      <c r="C684" s="4">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="685" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A685" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="B685" s="3"/>
+      <c r="C685" s="4"/>
+    </row>
+    <row r="686" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A686" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="B686" s="3"/>
+      <c r="C686" s="4"/>
+    </row>
+    <row r="687" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A687" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="B687" s="3">
+        <v>31</v>
+      </c>
+      <c r="C687" s="4">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="688" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A688" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="B688" s="3"/>
+      <c r="C688" s="4"/>
+    </row>
+    <row r="689" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A689" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="B689" s="3"/>
+      <c r="C689" s="4"/>
+    </row>
+    <row r="690" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A690" s="1" t="s">
+        <v>609</v>
+      </c>
+      <c r="B690" s="3">
+        <v>8</v>
+      </c>
+      <c r="C690" s="4">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="691" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A691" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="B691" s="3"/>
+      <c r="C691" s="4"/>
+    </row>
+    <row r="692" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A692" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="B692" s="3"/>
+      <c r="C692" s="4"/>
+    </row>
+    <row r="693" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A693" s="1" t="s">
+        <v>612</v>
+      </c>
+      <c r="B693" s="3">
+        <v>8</v>
+      </c>
+      <c r="C693" s="4">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="694" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A694" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B694" s="3"/>
+      <c r="C694" s="4"/>
+    </row>
+    <row r="695" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A695" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="B695" s="3"/>
+      <c r="C695" s="4"/>
+    </row>
+    <row r="696" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A696" s="1" t="s">
+        <v>615</v>
+      </c>
+      <c r="B696" s="3">
+        <v>2</v>
+      </c>
+      <c r="C696" s="4">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="697" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A697" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="B697" s="3"/>
+      <c r="C697" s="4"/>
+    </row>
+    <row r="698" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A698" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="B698" s="3"/>
+      <c r="C698" s="4"/>
+    </row>
+    <row r="699" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A699" s="1" t="s">
+        <v>618</v>
+      </c>
+      <c r="B699" s="3"/>
+      <c r="C699" s="4">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="700" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A700" s="2" t="s">
+        <v>619</v>
+      </c>
+      <c r="B700" s="3"/>
+      <c r="C700" s="4"/>
+    </row>
+    <row r="701" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A701" s="2" t="s">
+        <v>620</v>
+      </c>
+      <c r="B701" s="3"/>
+      <c r="C701" s="4"/>
+    </row>
+    <row r="702" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A702" s="1" t="s">
+        <v>621</v>
+      </c>
+      <c r="B702" s="3"/>
+      <c r="C702" s="4">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="703" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A703" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="B703" s="3"/>
+      <c r="C703" s="4"/>
+    </row>
+    <row r="704" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A704" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="B704" s="3"/>
+      <c r="C704" s="4"/>
+    </row>
+    <row r="705" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A705" s="1" t="s">
+        <v>624</v>
+      </c>
+      <c r="B705" s="3"/>
+      <c r="C705" s="4">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="706" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A706" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="B706" s="3"/>
+      <c r="C706" s="4"/>
+    </row>
+    <row r="707" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A707" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B707" s="3"/>
+      <c r="C707" s="4"/>
+    </row>
+    <row r="708" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A708" s="1" t="s">
+        <v>627</v>
+      </c>
+      <c r="B708" s="3"/>
+      <c r="C708" s="4">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="709" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A709" s="2" t="s">
+        <v>628</v>
+      </c>
+      <c r="B709" s="3"/>
+      <c r="C709" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="376">
-    <mergeCell ref="B556:B557"/>
-    <mergeCell ref="C556:C557"/>
-    <mergeCell ref="B558:B560"/>
-    <mergeCell ref="C558:C560"/>
-    <mergeCell ref="B548:B550"/>
-    <mergeCell ref="C548:C550"/>
-    <mergeCell ref="B551:B552"/>
-    <mergeCell ref="C551:C552"/>
-    <mergeCell ref="B553:B555"/>
-    <mergeCell ref="C553:C555"/>
+  <mergeCells count="478">
+    <mergeCell ref="B699:B701"/>
+    <mergeCell ref="C699:C701"/>
+    <mergeCell ref="B702:B704"/>
+    <mergeCell ref="C702:C704"/>
+    <mergeCell ref="B705:B707"/>
+    <mergeCell ref="C705:C707"/>
+    <mergeCell ref="B708:B709"/>
+    <mergeCell ref="C708:C709"/>
+    <mergeCell ref="B684:B686"/>
+    <mergeCell ref="C684:C686"/>
+    <mergeCell ref="B687:B689"/>
+    <mergeCell ref="C687:C689"/>
+    <mergeCell ref="B690:B692"/>
+    <mergeCell ref="C690:C692"/>
+    <mergeCell ref="B693:B695"/>
+    <mergeCell ref="C693:C695"/>
+    <mergeCell ref="B696:B698"/>
+    <mergeCell ref="C696:C698"/>
+    <mergeCell ref="B670:B672"/>
+    <mergeCell ref="C670:C672"/>
+    <mergeCell ref="B673:B675"/>
+    <mergeCell ref="C673:C675"/>
+    <mergeCell ref="B676:B678"/>
+    <mergeCell ref="C676:C678"/>
+    <mergeCell ref="B679:B680"/>
+    <mergeCell ref="C679:C680"/>
+    <mergeCell ref="B681:B683"/>
+    <mergeCell ref="C681:C683"/>
+    <mergeCell ref="B655:B657"/>
+    <mergeCell ref="C655:C657"/>
+    <mergeCell ref="B658:B660"/>
+    <mergeCell ref="C658:C660"/>
+    <mergeCell ref="B661:B663"/>
+    <mergeCell ref="C661:C663"/>
+    <mergeCell ref="B664:B666"/>
+    <mergeCell ref="C664:C666"/>
+    <mergeCell ref="B667:B669"/>
+    <mergeCell ref="C667:C669"/>
+    <mergeCell ref="B640:B642"/>
+    <mergeCell ref="C640:C642"/>
+    <mergeCell ref="B643:B645"/>
+    <mergeCell ref="C643:C645"/>
+    <mergeCell ref="B646:B648"/>
+    <mergeCell ref="C646:C648"/>
+    <mergeCell ref="B649:B651"/>
+    <mergeCell ref="C649:C651"/>
+    <mergeCell ref="B652:B654"/>
+    <mergeCell ref="C652:C654"/>
+    <mergeCell ref="B625:B627"/>
+    <mergeCell ref="C625:C627"/>
+    <mergeCell ref="B628:B630"/>
+    <mergeCell ref="C628:C630"/>
+    <mergeCell ref="B631:B633"/>
+    <mergeCell ref="C631:C633"/>
+    <mergeCell ref="B634:B636"/>
+    <mergeCell ref="C634:C636"/>
+    <mergeCell ref="B637:B639"/>
+    <mergeCell ref="C637:C639"/>
+    <mergeCell ref="B610:B612"/>
+    <mergeCell ref="C610:C612"/>
+    <mergeCell ref="B613:B615"/>
+    <mergeCell ref="C613:C615"/>
+    <mergeCell ref="B616:B618"/>
+    <mergeCell ref="C616:C618"/>
+    <mergeCell ref="B619:B621"/>
+    <mergeCell ref="C619:C621"/>
+    <mergeCell ref="B622:B624"/>
+    <mergeCell ref="C622:C624"/>
+    <mergeCell ref="B597:B599"/>
+    <mergeCell ref="C597:C599"/>
+    <mergeCell ref="B600:B601"/>
+    <mergeCell ref="C600:C601"/>
+    <mergeCell ref="B602:B604"/>
+    <mergeCell ref="C602:C604"/>
+    <mergeCell ref="B605:B607"/>
+    <mergeCell ref="C605:C607"/>
+    <mergeCell ref="B608:B609"/>
+    <mergeCell ref="C608:C609"/>
+    <mergeCell ref="B582:B584"/>
+    <mergeCell ref="C582:C584"/>
+    <mergeCell ref="B585:B587"/>
+    <mergeCell ref="C585:C587"/>
+    <mergeCell ref="B588:B590"/>
+    <mergeCell ref="C588:C590"/>
+    <mergeCell ref="B591:B593"/>
+    <mergeCell ref="C591:C593"/>
+    <mergeCell ref="B594:B596"/>
+    <mergeCell ref="C594:C596"/>
+    <mergeCell ref="B567:B569"/>
+    <mergeCell ref="C567:C569"/>
+    <mergeCell ref="B570:B572"/>
+    <mergeCell ref="C570:C572"/>
+    <mergeCell ref="B573:B575"/>
+    <mergeCell ref="C573:C575"/>
+    <mergeCell ref="B576:B578"/>
+    <mergeCell ref="C576:C578"/>
+    <mergeCell ref="B579:B581"/>
+    <mergeCell ref="C579:C581"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="B561:B563"/>
+    <mergeCell ref="C561:C563"/>
+    <mergeCell ref="B564:B566"/>
+    <mergeCell ref="C564:C566"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="B37:B39"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="B40:B42"/>
+    <mergeCell ref="C40:C42"/>
+    <mergeCell ref="B43:B45"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="C34:C36"/>
+    <mergeCell ref="B55:B57"/>
+    <mergeCell ref="C55:C57"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="C58:C60"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="C61:C63"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="B49:B51"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="B52:B54"/>
+    <mergeCell ref="C52:C54"/>
+    <mergeCell ref="B73:B75"/>
+    <mergeCell ref="C73:C75"/>
+    <mergeCell ref="B76:B78"/>
+    <mergeCell ref="C76:C78"/>
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="C79:C81"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="C64:C66"/>
+    <mergeCell ref="B67:B69"/>
+    <mergeCell ref="C67:C69"/>
+    <mergeCell ref="B70:B72"/>
+    <mergeCell ref="C70:C72"/>
+    <mergeCell ref="B91:B93"/>
+    <mergeCell ref="C91:C93"/>
+    <mergeCell ref="B94:B96"/>
+    <mergeCell ref="C94:C96"/>
+    <mergeCell ref="B97:B99"/>
+    <mergeCell ref="C97:C99"/>
+    <mergeCell ref="B82:B84"/>
+    <mergeCell ref="C82:C84"/>
+    <mergeCell ref="B85:B87"/>
+    <mergeCell ref="C85:C87"/>
+    <mergeCell ref="B88:B90"/>
+    <mergeCell ref="C88:C90"/>
+    <mergeCell ref="B109:B111"/>
+    <mergeCell ref="C109:C111"/>
+    <mergeCell ref="B112:B114"/>
+    <mergeCell ref="C112:C114"/>
+    <mergeCell ref="B115:B117"/>
+    <mergeCell ref="C115:C117"/>
+    <mergeCell ref="B100:B102"/>
+    <mergeCell ref="C100:C102"/>
+    <mergeCell ref="B103:B105"/>
+    <mergeCell ref="C103:C105"/>
+    <mergeCell ref="B106:B108"/>
+    <mergeCell ref="C106:C108"/>
+    <mergeCell ref="B127:B129"/>
+    <mergeCell ref="C127:C129"/>
+    <mergeCell ref="B130:B132"/>
+    <mergeCell ref="C130:C132"/>
+    <mergeCell ref="B133:B135"/>
+    <mergeCell ref="C133:C135"/>
+    <mergeCell ref="B118:B120"/>
+    <mergeCell ref="C118:C120"/>
+    <mergeCell ref="B121:B123"/>
+    <mergeCell ref="C121:C123"/>
+    <mergeCell ref="B124:B126"/>
+    <mergeCell ref="C124:C126"/>
+    <mergeCell ref="B145:B147"/>
+    <mergeCell ref="C145:C147"/>
+    <mergeCell ref="B148:B150"/>
+    <mergeCell ref="C148:C150"/>
+    <mergeCell ref="B151:B153"/>
+    <mergeCell ref="C151:C153"/>
+    <mergeCell ref="B136:B138"/>
+    <mergeCell ref="C136:C138"/>
+    <mergeCell ref="B139:B141"/>
+    <mergeCell ref="C139:C141"/>
+    <mergeCell ref="B142:B144"/>
+    <mergeCell ref="C142:C144"/>
+    <mergeCell ref="B163:B165"/>
+    <mergeCell ref="C163:C165"/>
+    <mergeCell ref="B166:B168"/>
+    <mergeCell ref="C166:C168"/>
+    <mergeCell ref="B169:B171"/>
+    <mergeCell ref="C169:C171"/>
+    <mergeCell ref="B154:B156"/>
+    <mergeCell ref="C154:C156"/>
+    <mergeCell ref="B157:B159"/>
+    <mergeCell ref="C157:C159"/>
+    <mergeCell ref="B160:B162"/>
+    <mergeCell ref="C160:C162"/>
+    <mergeCell ref="B181:B183"/>
+    <mergeCell ref="C181:C183"/>
+    <mergeCell ref="B184:B186"/>
+    <mergeCell ref="C184:C186"/>
+    <mergeCell ref="B187:B189"/>
+    <mergeCell ref="C187:C189"/>
+    <mergeCell ref="B172:B174"/>
+    <mergeCell ref="C172:C174"/>
+    <mergeCell ref="B175:B177"/>
+    <mergeCell ref="C175:C177"/>
+    <mergeCell ref="B178:B180"/>
+    <mergeCell ref="C178:C180"/>
+    <mergeCell ref="B199:B201"/>
+    <mergeCell ref="C199:C201"/>
+    <mergeCell ref="B202:B204"/>
+    <mergeCell ref="C202:C204"/>
+    <mergeCell ref="B205:B207"/>
+    <mergeCell ref="C205:C207"/>
+    <mergeCell ref="B190:B192"/>
+    <mergeCell ref="C190:C192"/>
+    <mergeCell ref="B193:B195"/>
+    <mergeCell ref="C193:C195"/>
+    <mergeCell ref="B196:B198"/>
+    <mergeCell ref="C196:C198"/>
+    <mergeCell ref="B217:B219"/>
+    <mergeCell ref="C217:C219"/>
+    <mergeCell ref="B220:B222"/>
+    <mergeCell ref="C220:C222"/>
+    <mergeCell ref="B223:B225"/>
+    <mergeCell ref="C223:C225"/>
+    <mergeCell ref="B208:B210"/>
+    <mergeCell ref="C208:C210"/>
+    <mergeCell ref="B211:B213"/>
+    <mergeCell ref="C211:C213"/>
+    <mergeCell ref="B214:B216"/>
+    <mergeCell ref="C214:C216"/>
+    <mergeCell ref="B235:B237"/>
+    <mergeCell ref="C235:C237"/>
+    <mergeCell ref="B238:B240"/>
+    <mergeCell ref="C238:C240"/>
+    <mergeCell ref="B241:B243"/>
+    <mergeCell ref="C241:C243"/>
+    <mergeCell ref="B226:B228"/>
+    <mergeCell ref="C226:C228"/>
+    <mergeCell ref="B229:B231"/>
+    <mergeCell ref="C229:C231"/>
+    <mergeCell ref="B232:B234"/>
+    <mergeCell ref="C232:C234"/>
+    <mergeCell ref="B253:B255"/>
+    <mergeCell ref="C253:C255"/>
+    <mergeCell ref="B256:B258"/>
+    <mergeCell ref="C256:C258"/>
+    <mergeCell ref="B259:B261"/>
+    <mergeCell ref="C259:C261"/>
+    <mergeCell ref="B244:B246"/>
+    <mergeCell ref="C244:C246"/>
+    <mergeCell ref="B247:B249"/>
+    <mergeCell ref="C247:C249"/>
+    <mergeCell ref="B250:B252"/>
+    <mergeCell ref="C250:C252"/>
+    <mergeCell ref="B271:B273"/>
+    <mergeCell ref="C271:C273"/>
+    <mergeCell ref="B274:B276"/>
+    <mergeCell ref="C274:C276"/>
+    <mergeCell ref="B277:B279"/>
+    <mergeCell ref="C277:C279"/>
+    <mergeCell ref="B262:B264"/>
+    <mergeCell ref="C262:C264"/>
+    <mergeCell ref="B265:B267"/>
+    <mergeCell ref="C265:C267"/>
+    <mergeCell ref="B268:B270"/>
+    <mergeCell ref="C268:C270"/>
+    <mergeCell ref="B289:B291"/>
+    <mergeCell ref="C289:C291"/>
+    <mergeCell ref="B292:B294"/>
+    <mergeCell ref="C292:C294"/>
+    <mergeCell ref="B295:B297"/>
+    <mergeCell ref="C295:C297"/>
+    <mergeCell ref="B280:B282"/>
+    <mergeCell ref="C280:C282"/>
+    <mergeCell ref="B283:B285"/>
+    <mergeCell ref="C283:C285"/>
+    <mergeCell ref="B286:B288"/>
+    <mergeCell ref="C286:C288"/>
+    <mergeCell ref="B307:B309"/>
+    <mergeCell ref="C307:C309"/>
+    <mergeCell ref="B310:B312"/>
+    <mergeCell ref="C310:C312"/>
+    <mergeCell ref="B313:B315"/>
+    <mergeCell ref="C313:C315"/>
+    <mergeCell ref="B298:B300"/>
+    <mergeCell ref="C298:C300"/>
+    <mergeCell ref="B301:B303"/>
+    <mergeCell ref="C301:C303"/>
+    <mergeCell ref="B304:B306"/>
+    <mergeCell ref="C304:C306"/>
+    <mergeCell ref="B325:B327"/>
+    <mergeCell ref="C325:C327"/>
+    <mergeCell ref="B328:B330"/>
+    <mergeCell ref="C328:C330"/>
+    <mergeCell ref="B331:B333"/>
+    <mergeCell ref="C331:C333"/>
+    <mergeCell ref="B316:B318"/>
+    <mergeCell ref="C316:C318"/>
+    <mergeCell ref="B319:B321"/>
+    <mergeCell ref="C319:C321"/>
+    <mergeCell ref="B322:B324"/>
+    <mergeCell ref="C322:C324"/>
+    <mergeCell ref="B343:B345"/>
+    <mergeCell ref="C343:C345"/>
+    <mergeCell ref="B346:B348"/>
+    <mergeCell ref="C346:C348"/>
+    <mergeCell ref="B349:B351"/>
+    <mergeCell ref="C349:C351"/>
+    <mergeCell ref="B334:B336"/>
+    <mergeCell ref="C334:C336"/>
+    <mergeCell ref="B337:B339"/>
+    <mergeCell ref="C337:C339"/>
+    <mergeCell ref="B340:B342"/>
+    <mergeCell ref="C340:C342"/>
+    <mergeCell ref="B361:B363"/>
+    <mergeCell ref="C361:C363"/>
+    <mergeCell ref="B364:B366"/>
+    <mergeCell ref="C364:C366"/>
+    <mergeCell ref="B367:B369"/>
+    <mergeCell ref="C367:C369"/>
+    <mergeCell ref="B352:B354"/>
+    <mergeCell ref="C352:C354"/>
+    <mergeCell ref="B355:B357"/>
+    <mergeCell ref="C355:C357"/>
+    <mergeCell ref="B358:B360"/>
+    <mergeCell ref="C358:C360"/>
+    <mergeCell ref="B379:B381"/>
+    <mergeCell ref="C379:C381"/>
+    <mergeCell ref="B382:B384"/>
+    <mergeCell ref="C382:C384"/>
+    <mergeCell ref="B385:B387"/>
+    <mergeCell ref="C385:C387"/>
+    <mergeCell ref="B370:B372"/>
+    <mergeCell ref="C370:C372"/>
+    <mergeCell ref="B373:B375"/>
+    <mergeCell ref="C373:C375"/>
+    <mergeCell ref="B376:B378"/>
+    <mergeCell ref="C376:C378"/>
+    <mergeCell ref="B397:B399"/>
+    <mergeCell ref="C397:C399"/>
+    <mergeCell ref="B400:B402"/>
+    <mergeCell ref="C400:C402"/>
+    <mergeCell ref="B403:B405"/>
+    <mergeCell ref="C403:C405"/>
+    <mergeCell ref="B388:B390"/>
+    <mergeCell ref="C388:C390"/>
+    <mergeCell ref="B391:B393"/>
+    <mergeCell ref="C391:C393"/>
+    <mergeCell ref="B394:B396"/>
+    <mergeCell ref="C394:C396"/>
+    <mergeCell ref="B415:B417"/>
+    <mergeCell ref="C415:C417"/>
+    <mergeCell ref="B418:B420"/>
+    <mergeCell ref="C418:C420"/>
+    <mergeCell ref="B421:B423"/>
+    <mergeCell ref="C421:C423"/>
+    <mergeCell ref="B406:B408"/>
+    <mergeCell ref="C406:C408"/>
+    <mergeCell ref="B409:B411"/>
+    <mergeCell ref="C409:C411"/>
+    <mergeCell ref="B412:B414"/>
+    <mergeCell ref="C412:C414"/>
+    <mergeCell ref="B433:B435"/>
+    <mergeCell ref="C433:C435"/>
+    <mergeCell ref="B436:B438"/>
+    <mergeCell ref="C436:C438"/>
+    <mergeCell ref="B439:B441"/>
+    <mergeCell ref="C439:C441"/>
+    <mergeCell ref="B424:B426"/>
+    <mergeCell ref="C424:C426"/>
+    <mergeCell ref="B427:B429"/>
+    <mergeCell ref="C427:C429"/>
+    <mergeCell ref="B430:B432"/>
+    <mergeCell ref="C430:C432"/>
+    <mergeCell ref="B450:B452"/>
+    <mergeCell ref="C450:C452"/>
+    <mergeCell ref="B453:B455"/>
+    <mergeCell ref="C453:C455"/>
+    <mergeCell ref="B456:B458"/>
+    <mergeCell ref="C456:C458"/>
+    <mergeCell ref="B442:B444"/>
+    <mergeCell ref="C442:C444"/>
+    <mergeCell ref="B445:B447"/>
+    <mergeCell ref="C445:C447"/>
+    <mergeCell ref="B448:B449"/>
+    <mergeCell ref="C448:C449"/>
+    <mergeCell ref="B468:B470"/>
+    <mergeCell ref="C468:C470"/>
+    <mergeCell ref="B471:B473"/>
+    <mergeCell ref="C471:C473"/>
+    <mergeCell ref="B474:B476"/>
+    <mergeCell ref="C474:C476"/>
+    <mergeCell ref="B459:B461"/>
+    <mergeCell ref="C459:C461"/>
+    <mergeCell ref="B462:B464"/>
+    <mergeCell ref="C462:C464"/>
+    <mergeCell ref="B465:B467"/>
+    <mergeCell ref="C465:C467"/>
+    <mergeCell ref="B485:B487"/>
+    <mergeCell ref="C485:C487"/>
+    <mergeCell ref="B488:B490"/>
+    <mergeCell ref="C488:C490"/>
+    <mergeCell ref="B491:B493"/>
+    <mergeCell ref="C491:C493"/>
+    <mergeCell ref="B477:B479"/>
+    <mergeCell ref="C477:C479"/>
+    <mergeCell ref="B480:B482"/>
+    <mergeCell ref="C480:C482"/>
+    <mergeCell ref="B483:B484"/>
+    <mergeCell ref="C483:C484"/>
+    <mergeCell ref="B503:B505"/>
+    <mergeCell ref="C503:C505"/>
+    <mergeCell ref="B506:B508"/>
+    <mergeCell ref="C506:C508"/>
+    <mergeCell ref="B509:B511"/>
+    <mergeCell ref="C509:C511"/>
+    <mergeCell ref="B494:B496"/>
+    <mergeCell ref="C494:C496"/>
+    <mergeCell ref="B497:B499"/>
+    <mergeCell ref="C497:C499"/>
+    <mergeCell ref="B500:B502"/>
+    <mergeCell ref="C500:C502"/>
+    <mergeCell ref="B521:B523"/>
+    <mergeCell ref="C521:C523"/>
+    <mergeCell ref="B524:B526"/>
+    <mergeCell ref="C524:C526"/>
+    <mergeCell ref="B527:B529"/>
+    <mergeCell ref="C527:C529"/>
+    <mergeCell ref="B512:B514"/>
+    <mergeCell ref="C512:C514"/>
+    <mergeCell ref="B515:B517"/>
+    <mergeCell ref="C515:C517"/>
+    <mergeCell ref="B518:B520"/>
+    <mergeCell ref="C518:C520"/>
     <mergeCell ref="B539:B541"/>
     <mergeCell ref="C539:C541"/>
     <mergeCell ref="B542:B544"/>
@@ -6709,360 +8715,16 @@
     <mergeCell ref="C533:C535"/>
     <mergeCell ref="B536:B538"/>
     <mergeCell ref="C536:C538"/>
-    <mergeCell ref="B521:B523"/>
-    <mergeCell ref="C521:C523"/>
-    <mergeCell ref="B524:B526"/>
-    <mergeCell ref="C524:C526"/>
-    <mergeCell ref="B527:B529"/>
-    <mergeCell ref="C527:C529"/>
-    <mergeCell ref="B512:B514"/>
-    <mergeCell ref="C512:C514"/>
-    <mergeCell ref="B515:B517"/>
-    <mergeCell ref="C515:C517"/>
-    <mergeCell ref="B518:B520"/>
-    <mergeCell ref="C518:C520"/>
-    <mergeCell ref="B503:B505"/>
-    <mergeCell ref="C503:C505"/>
-    <mergeCell ref="B506:B508"/>
-    <mergeCell ref="C506:C508"/>
-    <mergeCell ref="B509:B511"/>
-    <mergeCell ref="C509:C511"/>
-    <mergeCell ref="B494:B496"/>
-    <mergeCell ref="C494:C496"/>
-    <mergeCell ref="B497:B499"/>
-    <mergeCell ref="C497:C499"/>
-    <mergeCell ref="B500:B502"/>
-    <mergeCell ref="C500:C502"/>
-    <mergeCell ref="B485:B487"/>
-    <mergeCell ref="C485:C487"/>
-    <mergeCell ref="B488:B490"/>
-    <mergeCell ref="C488:C490"/>
-    <mergeCell ref="B491:B493"/>
-    <mergeCell ref="C491:C493"/>
-    <mergeCell ref="B477:B479"/>
-    <mergeCell ref="C477:C479"/>
-    <mergeCell ref="B480:B482"/>
-    <mergeCell ref="C480:C482"/>
-    <mergeCell ref="B483:B484"/>
-    <mergeCell ref="C483:C484"/>
-    <mergeCell ref="B468:B470"/>
-    <mergeCell ref="C468:C470"/>
-    <mergeCell ref="B471:B473"/>
-    <mergeCell ref="C471:C473"/>
-    <mergeCell ref="B474:B476"/>
-    <mergeCell ref="C474:C476"/>
-    <mergeCell ref="B459:B461"/>
-    <mergeCell ref="C459:C461"/>
-    <mergeCell ref="B462:B464"/>
-    <mergeCell ref="C462:C464"/>
-    <mergeCell ref="B465:B467"/>
-    <mergeCell ref="C465:C467"/>
-    <mergeCell ref="B450:B452"/>
-    <mergeCell ref="C450:C452"/>
-    <mergeCell ref="B453:B455"/>
-    <mergeCell ref="C453:C455"/>
-    <mergeCell ref="B456:B458"/>
-    <mergeCell ref="C456:C458"/>
-    <mergeCell ref="B442:B444"/>
-    <mergeCell ref="C442:C444"/>
-    <mergeCell ref="B445:B447"/>
-    <mergeCell ref="C445:C447"/>
-    <mergeCell ref="B448:B449"/>
-    <mergeCell ref="C448:C449"/>
-    <mergeCell ref="B433:B435"/>
-    <mergeCell ref="C433:C435"/>
-    <mergeCell ref="B436:B438"/>
-    <mergeCell ref="C436:C438"/>
-    <mergeCell ref="B439:B441"/>
-    <mergeCell ref="C439:C441"/>
-    <mergeCell ref="B424:B426"/>
-    <mergeCell ref="C424:C426"/>
-    <mergeCell ref="B427:B429"/>
-    <mergeCell ref="C427:C429"/>
-    <mergeCell ref="B430:B432"/>
-    <mergeCell ref="C430:C432"/>
-    <mergeCell ref="B415:B417"/>
-    <mergeCell ref="C415:C417"/>
-    <mergeCell ref="B418:B420"/>
-    <mergeCell ref="C418:C420"/>
-    <mergeCell ref="B421:B423"/>
-    <mergeCell ref="C421:C423"/>
-    <mergeCell ref="B406:B408"/>
-    <mergeCell ref="C406:C408"/>
-    <mergeCell ref="B409:B411"/>
-    <mergeCell ref="C409:C411"/>
-    <mergeCell ref="B412:B414"/>
-    <mergeCell ref="C412:C414"/>
-    <mergeCell ref="B397:B399"/>
-    <mergeCell ref="C397:C399"/>
-    <mergeCell ref="B400:B402"/>
-    <mergeCell ref="C400:C402"/>
-    <mergeCell ref="B403:B405"/>
-    <mergeCell ref="C403:C405"/>
-    <mergeCell ref="B388:B390"/>
-    <mergeCell ref="C388:C390"/>
-    <mergeCell ref="B391:B393"/>
-    <mergeCell ref="C391:C393"/>
-    <mergeCell ref="B394:B396"/>
-    <mergeCell ref="C394:C396"/>
-    <mergeCell ref="B379:B381"/>
-    <mergeCell ref="C379:C381"/>
-    <mergeCell ref="B382:B384"/>
-    <mergeCell ref="C382:C384"/>
-    <mergeCell ref="B385:B387"/>
-    <mergeCell ref="C385:C387"/>
-    <mergeCell ref="B370:B372"/>
-    <mergeCell ref="C370:C372"/>
-    <mergeCell ref="B373:B375"/>
-    <mergeCell ref="C373:C375"/>
-    <mergeCell ref="B376:B378"/>
-    <mergeCell ref="C376:C378"/>
-    <mergeCell ref="B361:B363"/>
-    <mergeCell ref="C361:C363"/>
-    <mergeCell ref="B364:B366"/>
-    <mergeCell ref="C364:C366"/>
-    <mergeCell ref="B367:B369"/>
-    <mergeCell ref="C367:C369"/>
-    <mergeCell ref="B352:B354"/>
-    <mergeCell ref="C352:C354"/>
-    <mergeCell ref="B355:B357"/>
-    <mergeCell ref="C355:C357"/>
-    <mergeCell ref="B358:B360"/>
-    <mergeCell ref="C358:C360"/>
-    <mergeCell ref="B343:B345"/>
-    <mergeCell ref="C343:C345"/>
-    <mergeCell ref="B346:B348"/>
-    <mergeCell ref="C346:C348"/>
-    <mergeCell ref="B349:B351"/>
-    <mergeCell ref="C349:C351"/>
-    <mergeCell ref="B334:B336"/>
-    <mergeCell ref="C334:C336"/>
-    <mergeCell ref="B337:B339"/>
-    <mergeCell ref="C337:C339"/>
-    <mergeCell ref="B340:B342"/>
-    <mergeCell ref="C340:C342"/>
-    <mergeCell ref="B325:B327"/>
-    <mergeCell ref="C325:C327"/>
-    <mergeCell ref="B328:B330"/>
-    <mergeCell ref="C328:C330"/>
-    <mergeCell ref="B331:B333"/>
-    <mergeCell ref="C331:C333"/>
-    <mergeCell ref="B316:B318"/>
-    <mergeCell ref="C316:C318"/>
-    <mergeCell ref="B319:B321"/>
-    <mergeCell ref="C319:C321"/>
-    <mergeCell ref="B322:B324"/>
-    <mergeCell ref="C322:C324"/>
-    <mergeCell ref="B307:B309"/>
-    <mergeCell ref="C307:C309"/>
-    <mergeCell ref="B310:B312"/>
-    <mergeCell ref="C310:C312"/>
-    <mergeCell ref="B313:B315"/>
-    <mergeCell ref="C313:C315"/>
-    <mergeCell ref="B298:B300"/>
-    <mergeCell ref="C298:C300"/>
-    <mergeCell ref="B301:B303"/>
-    <mergeCell ref="C301:C303"/>
-    <mergeCell ref="B304:B306"/>
-    <mergeCell ref="C304:C306"/>
-    <mergeCell ref="B289:B291"/>
-    <mergeCell ref="C289:C291"/>
-    <mergeCell ref="B292:B294"/>
-    <mergeCell ref="C292:C294"/>
-    <mergeCell ref="B295:B297"/>
-    <mergeCell ref="C295:C297"/>
-    <mergeCell ref="B280:B282"/>
-    <mergeCell ref="C280:C282"/>
-    <mergeCell ref="B283:B285"/>
-    <mergeCell ref="C283:C285"/>
-    <mergeCell ref="B286:B288"/>
-    <mergeCell ref="C286:C288"/>
-    <mergeCell ref="B271:B273"/>
-    <mergeCell ref="C271:C273"/>
-    <mergeCell ref="B274:B276"/>
-    <mergeCell ref="C274:C276"/>
-    <mergeCell ref="B277:B279"/>
-    <mergeCell ref="C277:C279"/>
-    <mergeCell ref="B262:B264"/>
-    <mergeCell ref="C262:C264"/>
-    <mergeCell ref="B265:B267"/>
-    <mergeCell ref="C265:C267"/>
-    <mergeCell ref="B268:B270"/>
-    <mergeCell ref="C268:C270"/>
-    <mergeCell ref="B253:B255"/>
-    <mergeCell ref="C253:C255"/>
-    <mergeCell ref="B256:B258"/>
-    <mergeCell ref="C256:C258"/>
-    <mergeCell ref="B259:B261"/>
-    <mergeCell ref="C259:C261"/>
-    <mergeCell ref="B244:B246"/>
-    <mergeCell ref="C244:C246"/>
-    <mergeCell ref="B247:B249"/>
-    <mergeCell ref="C247:C249"/>
-    <mergeCell ref="B250:B252"/>
-    <mergeCell ref="C250:C252"/>
-    <mergeCell ref="B235:B237"/>
-    <mergeCell ref="C235:C237"/>
-    <mergeCell ref="B238:B240"/>
-    <mergeCell ref="C238:C240"/>
-    <mergeCell ref="B241:B243"/>
-    <mergeCell ref="C241:C243"/>
-    <mergeCell ref="B226:B228"/>
-    <mergeCell ref="C226:C228"/>
-    <mergeCell ref="B229:B231"/>
-    <mergeCell ref="C229:C231"/>
-    <mergeCell ref="B232:B234"/>
-    <mergeCell ref="C232:C234"/>
-    <mergeCell ref="B217:B219"/>
-    <mergeCell ref="C217:C219"/>
-    <mergeCell ref="B220:B222"/>
-    <mergeCell ref="C220:C222"/>
-    <mergeCell ref="B223:B225"/>
-    <mergeCell ref="C223:C225"/>
-    <mergeCell ref="B208:B210"/>
-    <mergeCell ref="C208:C210"/>
-    <mergeCell ref="B211:B213"/>
-    <mergeCell ref="C211:C213"/>
-    <mergeCell ref="B214:B216"/>
-    <mergeCell ref="C214:C216"/>
-    <mergeCell ref="B199:B201"/>
-    <mergeCell ref="C199:C201"/>
-    <mergeCell ref="B202:B204"/>
-    <mergeCell ref="C202:C204"/>
-    <mergeCell ref="B205:B207"/>
-    <mergeCell ref="C205:C207"/>
-    <mergeCell ref="B190:B192"/>
-    <mergeCell ref="C190:C192"/>
-    <mergeCell ref="B193:B195"/>
-    <mergeCell ref="C193:C195"/>
-    <mergeCell ref="B196:B198"/>
-    <mergeCell ref="C196:C198"/>
-    <mergeCell ref="B181:B183"/>
-    <mergeCell ref="C181:C183"/>
-    <mergeCell ref="B184:B186"/>
-    <mergeCell ref="C184:C186"/>
-    <mergeCell ref="B187:B189"/>
-    <mergeCell ref="C187:C189"/>
-    <mergeCell ref="B172:B174"/>
-    <mergeCell ref="C172:C174"/>
-    <mergeCell ref="B175:B177"/>
-    <mergeCell ref="C175:C177"/>
-    <mergeCell ref="B178:B180"/>
-    <mergeCell ref="C178:C180"/>
-    <mergeCell ref="B163:B165"/>
-    <mergeCell ref="C163:C165"/>
-    <mergeCell ref="B166:B168"/>
-    <mergeCell ref="C166:C168"/>
-    <mergeCell ref="B169:B171"/>
-    <mergeCell ref="C169:C171"/>
-    <mergeCell ref="B154:B156"/>
-    <mergeCell ref="C154:C156"/>
-    <mergeCell ref="B157:B159"/>
-    <mergeCell ref="C157:C159"/>
-    <mergeCell ref="B160:B162"/>
-    <mergeCell ref="C160:C162"/>
-    <mergeCell ref="B145:B147"/>
-    <mergeCell ref="C145:C147"/>
-    <mergeCell ref="B148:B150"/>
-    <mergeCell ref="C148:C150"/>
-    <mergeCell ref="B151:B153"/>
-    <mergeCell ref="C151:C153"/>
-    <mergeCell ref="B136:B138"/>
-    <mergeCell ref="C136:C138"/>
-    <mergeCell ref="B139:B141"/>
-    <mergeCell ref="C139:C141"/>
-    <mergeCell ref="B142:B144"/>
-    <mergeCell ref="C142:C144"/>
-    <mergeCell ref="B127:B129"/>
-    <mergeCell ref="C127:C129"/>
-    <mergeCell ref="B130:B132"/>
-    <mergeCell ref="C130:C132"/>
-    <mergeCell ref="B133:B135"/>
-    <mergeCell ref="C133:C135"/>
-    <mergeCell ref="B118:B120"/>
-    <mergeCell ref="C118:C120"/>
-    <mergeCell ref="B121:B123"/>
-    <mergeCell ref="C121:C123"/>
-    <mergeCell ref="B124:B126"/>
-    <mergeCell ref="C124:C126"/>
-    <mergeCell ref="B109:B111"/>
-    <mergeCell ref="C109:C111"/>
-    <mergeCell ref="B112:B114"/>
-    <mergeCell ref="C112:C114"/>
-    <mergeCell ref="B115:B117"/>
-    <mergeCell ref="C115:C117"/>
-    <mergeCell ref="B100:B102"/>
-    <mergeCell ref="C100:C102"/>
-    <mergeCell ref="B103:B105"/>
-    <mergeCell ref="C103:C105"/>
-    <mergeCell ref="B106:B108"/>
-    <mergeCell ref="C106:C108"/>
-    <mergeCell ref="B91:B93"/>
-    <mergeCell ref="C91:C93"/>
-    <mergeCell ref="B94:B96"/>
-    <mergeCell ref="C94:C96"/>
-    <mergeCell ref="B97:B99"/>
-    <mergeCell ref="C97:C99"/>
-    <mergeCell ref="B82:B84"/>
-    <mergeCell ref="C82:C84"/>
-    <mergeCell ref="B85:B87"/>
-    <mergeCell ref="C85:C87"/>
-    <mergeCell ref="B88:B90"/>
-    <mergeCell ref="C88:C90"/>
-    <mergeCell ref="B73:B75"/>
-    <mergeCell ref="C73:C75"/>
-    <mergeCell ref="B76:B78"/>
-    <mergeCell ref="C76:C78"/>
-    <mergeCell ref="B79:B81"/>
-    <mergeCell ref="C79:C81"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="C64:C66"/>
-    <mergeCell ref="B67:B69"/>
-    <mergeCell ref="C67:C69"/>
-    <mergeCell ref="B70:B72"/>
-    <mergeCell ref="C70:C72"/>
-    <mergeCell ref="B55:B57"/>
-    <mergeCell ref="C55:C57"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="C58:C60"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="C61:C63"/>
-    <mergeCell ref="B46:B48"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="B49:B51"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="B52:B54"/>
-    <mergeCell ref="C52:C54"/>
-    <mergeCell ref="B37:B39"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="B40:B42"/>
-    <mergeCell ref="C40:C42"/>
-    <mergeCell ref="B43:B45"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="C31:C33"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="C34:C36"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="C19:C21"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="C22:C24"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="C25:C27"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="B556:B557"/>
+    <mergeCell ref="C556:C557"/>
+    <mergeCell ref="B558:B560"/>
+    <mergeCell ref="C558:C560"/>
+    <mergeCell ref="B548:B550"/>
+    <mergeCell ref="C548:C550"/>
+    <mergeCell ref="B551:B552"/>
+    <mergeCell ref="C551:C552"/>
+    <mergeCell ref="B553:B555"/>
+    <mergeCell ref="C553:C555"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" r:id="rId1" display="https://scholar.google.ca/citations?view_op=view_citation&amp;hl=en&amp;user=lotIW94AAAAJ&amp;citation_for_view=lotIW94AAAAJ:xtRiw3GOFMkC" xr:uid="{0E1A47C0-B24F-A547-B175-807B2A556D7E}"/>
@@ -7436,6 +9098,107 @@
     <hyperlink ref="B556" r:id="rId340" display="https://scholar.google.ca/scholar?oi=bibs&amp;hl=en&amp;cites=9513485110243366275" xr:uid="{EA64D2E5-0267-F541-A023-B046287144CA}"/>
     <hyperlink ref="A558" r:id="rId341" display="https://scholar.google.ca/citations?view_op=view_citation&amp;hl=en&amp;user=gJ4oeJEAAAAJ&amp;citation_for_view=gJ4oeJEAAAAJ:d1gkVwhDpl0C" xr:uid="{F20E747C-AD44-374A-A35B-4ED1CFA0451A}"/>
     <hyperlink ref="B558" r:id="rId342" display="https://scholar.google.ca/scholar?oi=bibs&amp;hl=en&amp;cites=13387262746893670169" xr:uid="{BA87B8EC-DE94-344C-9678-0484D3591908}"/>
+    <hyperlink ref="A561" r:id="rId343" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:2osOgNQ5qMEC" xr:uid="{38323CF8-6FB9-A346-9004-9BCCB5D1ADF1}"/>
+    <hyperlink ref="B561" r:id="rId344" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=18438821309036428096" xr:uid="{4D227B07-A2DA-8440-8BF4-F1CD707B6767}"/>
+    <hyperlink ref="A564" r:id="rId345" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:9yKSN-GCB0IC" xr:uid="{7A2429BB-E8D8-1545-9615-C85E07B53FF3}"/>
+    <hyperlink ref="B564" r:id="rId346" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=10199253588006063450" xr:uid="{AB810BA5-DB5E-514C-BB90-946C09DD2DF4}"/>
+    <hyperlink ref="A567" r:id="rId347" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:d1gkVwhDpl0C" xr:uid="{BC7D4E69-C0F1-234F-933A-3421060894AF}"/>
+    <hyperlink ref="B567" r:id="rId348" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=5394371955331720451,3464617528505037522" xr:uid="{8D45ADDF-E22F-B745-AB3A-968EFAB5F8F5}"/>
+    <hyperlink ref="A570" r:id="rId349" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:qjMakFHDy7sC" xr:uid="{299A71C5-9CA8-7E4C-A193-5CAC3B7419E5}"/>
+    <hyperlink ref="B570" r:id="rId350" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=14682916917507945538" xr:uid="{0B8F4095-47E6-344A-80D8-E2BC1221D175}"/>
+    <hyperlink ref="A573" r:id="rId351" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:3fE2CSJIrl8C" xr:uid="{2A84EDE8-57CD-4749-9B6B-34A80D7BFCA4}"/>
+    <hyperlink ref="B573" r:id="rId352" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=14518297721468927072" xr:uid="{A6EA550D-BE52-724E-B0C0-6BA07C8ADADA}"/>
+    <hyperlink ref="A576" r:id="rId353" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:5nxA0vEk-isC" xr:uid="{F7CEF5D7-6E09-924C-AC3E-E116821E97D9}"/>
+    <hyperlink ref="B576" r:id="rId354" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=15431931766288051897" xr:uid="{570C1D8E-D822-EC44-9C69-FA8813ECD00B}"/>
+    <hyperlink ref="A579" r:id="rId355" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:W7OEmFMy1HYC" xr:uid="{A9D54770-C7FE-084D-BA80-D4D7137E6CFC}"/>
+    <hyperlink ref="B579" r:id="rId356" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=15260255064978446488" xr:uid="{9137A70F-7B78-EC40-BFD7-D09C9C5838AF}"/>
+    <hyperlink ref="A582" r:id="rId357" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:UebtZRa9Y70C" xr:uid="{25C71EDA-279B-9842-8F38-F6E54234D0BD}"/>
+    <hyperlink ref="B582" r:id="rId358" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=12384977865030484821" xr:uid="{A8855B04-63B7-8D4A-B15A-BECFEAC1F118}"/>
+    <hyperlink ref="A585" r:id="rId359" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:Se3iqnhoufwC" xr:uid="{7737AD4C-2FEE-4544-BC03-6DCDDDA6AE7B}"/>
+    <hyperlink ref="B585" r:id="rId360" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=11478491708220273652" xr:uid="{EF67D154-1548-9A42-AF2C-5B7E91B39544}"/>
+    <hyperlink ref="A588" r:id="rId361" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:eQOLeE2rZwMC" xr:uid="{E6865631-5B53-A248-B7FD-6DB49D735DC4}"/>
+    <hyperlink ref="B588" r:id="rId362" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=445594232509227482" xr:uid="{E5B78B03-61C6-1545-B4AF-8D09DC1B8D57}"/>
+    <hyperlink ref="A591" r:id="rId363" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:Wp0gIr-vW9MC" xr:uid="{3DCC3FE4-B093-DC4C-9944-FB125D22C2DE}"/>
+    <hyperlink ref="B591" r:id="rId364" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=4599190040013596024" xr:uid="{5128CE87-B13B-2444-A3B6-093E5D21EACD}"/>
+    <hyperlink ref="A594" r:id="rId365" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:Zph67rFs4hoC" xr:uid="{03E06999-84A5-5042-952A-CB02E53CB311}"/>
+    <hyperlink ref="B594" r:id="rId366" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=17221536997697496231" xr:uid="{2A15D51D-47B1-8B47-8FA6-869EBFB720E1}"/>
+    <hyperlink ref="A597" r:id="rId367" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:-f6ydRqryjwC" xr:uid="{CDFAD303-BAE2-B64B-9312-16F9EF60DAD9}"/>
+    <hyperlink ref="B597" r:id="rId368" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=11247321173341005052" xr:uid="{031503EC-2C69-FF41-9758-8CF954D8D378}"/>
+    <hyperlink ref="A600" r:id="rId369" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:LkGwnXOMwfcC" xr:uid="{B690395B-D125-F44D-A06E-329C3B85D807}"/>
+    <hyperlink ref="B600" r:id="rId370" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=11765246759472421603" xr:uid="{D896DEB7-902C-284A-ACB4-0E8683869642}"/>
+    <hyperlink ref="A602" r:id="rId371" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:Y0pCki6q_DkC" xr:uid="{25227F6B-3550-DD46-A023-A96829CFC39E}"/>
+    <hyperlink ref="B602" r:id="rId372" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=17617524555772456740" xr:uid="{CAF87E98-7ADC-454D-8F27-FC97E11DED2E}"/>
+    <hyperlink ref="A605" r:id="rId373" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:4DMP91E08xMC" xr:uid="{A583228E-2B61-6B46-817E-E50216F43AAD}"/>
+    <hyperlink ref="B605" r:id="rId374" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=11258725931960264031" xr:uid="{5AFEE5B4-4986-0648-A588-656828B8B0AB}"/>
+    <hyperlink ref="A608" r:id="rId375" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:mB3voiENLucC" xr:uid="{DA0884F2-9A8E-4243-A737-07050EA84AEA}"/>
+    <hyperlink ref="B608" xr:uid="{92884CA6-7D93-9E48-9499-83EB4E87643C}"/>
+    <hyperlink ref="A610" r:id="rId376" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:hFOr9nPyWt4C" xr:uid="{51180FB2-E55E-3248-9CD0-35C6132512BB}"/>
+    <hyperlink ref="B610" xr:uid="{A411A3D8-449E-E64D-BAC3-8BFB7FA555AF}"/>
+    <hyperlink ref="A613" r:id="rId377" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:YOwf2qJgpHMC" xr:uid="{D35FCF3D-732F-6144-A326-66C013C26801}"/>
+    <hyperlink ref="B613" xr:uid="{8DBF1737-CE95-0241-AF67-31AEF5B4D4FB}"/>
+    <hyperlink ref="A616" r:id="rId378" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MajTI0kAAAAJ&amp;citation_for_view=MajTI0kAAAAJ:M3ejUd6NZC8C" xr:uid="{1AB2FAF2-6599-6744-85E7-0B4CA200039F}"/>
+    <hyperlink ref="B616" xr:uid="{941EF143-70B2-1543-B49C-0A32255D5826}"/>
+    <hyperlink ref="A619" r:id="rId379" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:_FxGoFyzp5QC" xr:uid="{04D3BF3D-AB71-6A43-8D99-C60D207B086A}"/>
+    <hyperlink ref="B619" r:id="rId380" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=14943949718996492241,9295283714574589860" xr:uid="{55107CCA-6BD3-7E41-A5CE-994E76862821}"/>
+    <hyperlink ref="A622" r:id="rId381" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:YsMSGLbcyi4C" xr:uid="{AF42615C-0A8D-984F-AE74-DF10DAAD2273}"/>
+    <hyperlink ref="B622" r:id="rId382" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=13162351343408260130" xr:uid="{F5D734A1-0A7F-6F4C-BE93-0103F3DFDB37}"/>
+    <hyperlink ref="A625" r:id="rId383" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:WF5omc3nYNoC" xr:uid="{7485BA4D-AA5B-CD49-9FDF-7E04AD014BD6}"/>
+    <hyperlink ref="B625" r:id="rId384" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=15445732360366845980,2096223136222651988" xr:uid="{34BBB573-C79F-CA42-AABB-58D30D5C343C}"/>
+    <hyperlink ref="A628" r:id="rId385" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:qjMakFHDy7sC" xr:uid="{99D9321F-A778-A346-A46D-704581189D38}"/>
+    <hyperlink ref="A631" r:id="rId386" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:2osOgNQ5qMEC" xr:uid="{AF0D195D-7C03-6A49-97A8-44E59FBA68D4}"/>
+    <hyperlink ref="B631" r:id="rId387" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=6892275663945815970" xr:uid="{3CC00941-739B-5B43-88C4-7E846ED67E12}"/>
+    <hyperlink ref="A634" r:id="rId388" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:u-x6o8ySG0sC" xr:uid="{6565E707-4911-A442-8AD3-87A69E8BF2FC}"/>
+    <hyperlink ref="B634" r:id="rId389" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=1505539922492679102" xr:uid="{B4FE0E29-BE24-4E4C-AFE2-8203AC8244B7}"/>
+    <hyperlink ref="A637" r:id="rId390" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:u5HHmVD_uO8C" xr:uid="{A1D9B95B-52AC-0945-92B4-2EE2A4A503B9}"/>
+    <hyperlink ref="B637" r:id="rId391" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=1195250452201948679" xr:uid="{B944A079-6782-D247-AC5F-8A2AF69D7DC6}"/>
+    <hyperlink ref="A640" r:id="rId392" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:W7OEmFMy1HYC" xr:uid="{2C3B0EDC-AE81-B945-800F-35ECE5619BB4}"/>
+    <hyperlink ref="B640" r:id="rId393" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=12347233027893450893,4081673723780999764" xr:uid="{B221B3C1-375D-4A4D-829A-54E7B330E941}"/>
+    <hyperlink ref="A643" r:id="rId394" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:Se3iqnhoufwC" xr:uid="{70A0535D-282F-E148-BA00-906BD07AB97E}"/>
+    <hyperlink ref="B643" r:id="rId395" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=5518562443997509835" xr:uid="{222FC3B5-6B0E-E649-A849-78FFD283A757}"/>
+    <hyperlink ref="A646" r:id="rId396" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:zYLM7Y9cAGgC" xr:uid="{CA351F20-8381-994E-8831-A6E18260BA8A}"/>
+    <hyperlink ref="B646" r:id="rId397" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=8639077744506763903" xr:uid="{0510EDE9-AF42-6D4B-8DE4-4E42197AAB05}"/>
+    <hyperlink ref="A649" r:id="rId398" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:UeHWp8X0CEIC" xr:uid="{34C7ED57-A208-2745-8BA4-90F1F2330EDA}"/>
+    <hyperlink ref="B649" r:id="rId399" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=8398362486471036782" xr:uid="{57213D3F-1450-E844-BA14-644B833B6092}"/>
+    <hyperlink ref="A652" r:id="rId400" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:hqOjcs7Dif8C" xr:uid="{76528754-7F41-7849-AC1E-C5F99255D85A}"/>
+    <hyperlink ref="B652" r:id="rId401" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=13676995628850696864" xr:uid="{C30E8D6E-4E28-2945-891F-276BB5FB5135}"/>
+    <hyperlink ref="A655" r:id="rId402" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:Y0pCki6q_DkC" xr:uid="{3ABE0018-5AB6-E14E-8CBD-F9A884C00A60}"/>
+    <hyperlink ref="B655" r:id="rId403" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=12214531268750987377" xr:uid="{4929D805-6EAF-3F49-A4BA-68F0E1B1D0BB}"/>
+    <hyperlink ref="A658" r:id="rId404" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:5nxA0vEk-isC" xr:uid="{90E49A5D-3A85-3540-8EB9-4EADDC127403}"/>
+    <hyperlink ref="B658" r:id="rId405" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=8557475709729251005" xr:uid="{3F327CF0-9A47-B044-A975-3E3FEF0351CE}"/>
+    <hyperlink ref="A661" r:id="rId406" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:UebtZRa9Y70C" xr:uid="{02CAF606-2149-0744-BAA5-8D9347D0968A}"/>
+    <hyperlink ref="B661" r:id="rId407" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=4390265008156162287" xr:uid="{ADE9C1A8-B8E6-4F48-BCD8-C12235519ECA}"/>
+    <hyperlink ref="A664" r:id="rId408" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:3fE2CSJIrl8C" xr:uid="{FD3ABF8A-A9F7-DE43-B440-EC98B0E16F94}"/>
+    <hyperlink ref="B664" xr:uid="{C971C95C-ABCD-8B40-8D81-F740BE830825}"/>
+    <hyperlink ref="A667" r:id="rId409" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:0EnyYjriUFMC" xr:uid="{3A9E737D-1822-464F-9091-E9B7BAF9DC84}"/>
+    <hyperlink ref="B667" xr:uid="{3599401A-8514-E44F-BD51-0451F08CE78E}"/>
+    <hyperlink ref="A670" r:id="rId410" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:8k81kl-MbHgC" xr:uid="{CD38D470-3A80-434D-9F5D-B3D7525E0800}"/>
+    <hyperlink ref="B670" xr:uid="{6C1056B1-5E2F-6D4D-AEE7-0C60A64A5887}"/>
+    <hyperlink ref="A673" r:id="rId411" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:Tyk-4Ss8FVUC" xr:uid="{C78D2281-E55B-C746-A139-425869A51446}"/>
+    <hyperlink ref="B673" xr:uid="{DCF8A146-9B7F-2349-B2D2-5F6EA72D4CA4}"/>
+    <hyperlink ref="A676" r:id="rId412" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;citation_for_view=MhVneNwAAAAJ:IjCSPb-OGe4C" xr:uid="{0D3A73C3-6304-A045-80F5-9105FED4A9D6}"/>
+    <hyperlink ref="B676" xr:uid="{8E4F6276-9FF3-1449-BE25-8AE55ED093A1}"/>
+    <hyperlink ref="A679" r:id="rId413" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=MhVneNwAAAAJ&amp;cstart=20&amp;pagesize=80&amp;citation_for_view=MhVneNwAAAAJ:ufrVoPGSRksC" xr:uid="{ADEAA86B-1406-FC4D-AD92-9B84A4AA5796}"/>
+    <hyperlink ref="B679" xr:uid="{8134520B-D207-1440-BF89-A7125B3B0847}"/>
+    <hyperlink ref="A681" r:id="rId414" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=dq0JfDcAAAAJ&amp;citation_for_view=dq0JfDcAAAAJ:IjCSPb-OGe4C" xr:uid="{57EBE04C-1694-DE4C-8F3E-541B3015BDB6}"/>
+    <hyperlink ref="B681" r:id="rId415" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=12125926802820743093" xr:uid="{D9668CC8-08E4-4942-BA77-2622EEB1CDE1}"/>
+    <hyperlink ref="A684" r:id="rId416" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=dq0JfDcAAAAJ&amp;citation_for_view=dq0JfDcAAAAJ:9yKSN-GCB0IC" xr:uid="{A367D32F-1923-8040-B461-F8624F16EB4F}"/>
+    <hyperlink ref="B684" r:id="rId417" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=7380889746393990269" xr:uid="{C5170D3E-8E00-F649-B907-168EE34CA7F2}"/>
+    <hyperlink ref="A687" r:id="rId418" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=dq0JfDcAAAAJ&amp;citation_for_view=dq0JfDcAAAAJ:d1gkVwhDpl0C" xr:uid="{336B9BA8-1FDF-3543-85D8-8ABDB1DBC7EA}"/>
+    <hyperlink ref="B687" r:id="rId419" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=895373070968311813" xr:uid="{F5A0C93E-407D-E945-B079-07A65DA11227}"/>
+    <hyperlink ref="A690" r:id="rId420" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=dq0JfDcAAAAJ&amp;citation_for_view=dq0JfDcAAAAJ:Y0pCki6q_DkC" xr:uid="{76322B4C-7C8D-6240-8BA6-C4320F2612C0}"/>
+    <hyperlink ref="B690" r:id="rId421" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=16759362408447206514" xr:uid="{04C2EAD0-53D9-5240-921A-A54CFDB8ADBE}"/>
+    <hyperlink ref="A693" r:id="rId422" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=dq0JfDcAAAAJ&amp;citation_for_view=dq0JfDcAAAAJ:qjMakFHDy7sC" xr:uid="{3B2E40B8-0DC3-BB43-81AA-2C6079D248D2}"/>
+    <hyperlink ref="B693" r:id="rId423" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=9327618205908924005" xr:uid="{059B5B34-4E5D-AC45-B735-B4D212FB981B}"/>
+    <hyperlink ref="A696" r:id="rId424" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=dq0JfDcAAAAJ&amp;citation_for_view=dq0JfDcAAAAJ:YsMSGLbcyi4C" xr:uid="{3101AD4B-BFB6-EC4D-BF89-D1BC73AE0F9A}"/>
+    <hyperlink ref="B696" r:id="rId425" display="https://scholar.google.com/scholar?oi=bibs&amp;hl=en&amp;cites=9572686037325897793" xr:uid="{C5866D2F-76D9-1A4E-A7DA-5A873A5A69D9}"/>
+    <hyperlink ref="A699" r:id="rId426" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=dq0JfDcAAAAJ&amp;citation_for_view=dq0JfDcAAAAJ:UeHWp8X0CEIC" xr:uid="{D00B9E9E-650E-9C44-AC72-E25A39FE49F2}"/>
+    <hyperlink ref="B699" xr:uid="{12A15543-E927-2749-B30A-99C906709ECF}"/>
+    <hyperlink ref="A702" r:id="rId427" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=dq0JfDcAAAAJ&amp;citation_for_view=dq0JfDcAAAAJ:u-x6o8ySG0sC" xr:uid="{0CAD1EB8-94D0-9648-9588-39AC16B81326}"/>
+    <hyperlink ref="B702" xr:uid="{934E254C-B7C1-C244-BC93-6F2069D5C9BD}"/>
+    <hyperlink ref="A705" r:id="rId428" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=dq0JfDcAAAAJ&amp;citation_for_view=dq0JfDcAAAAJ:W7OEmFMy1HYC" xr:uid="{DC91BC4F-630B-A148-8FF6-7D9F2AD5016D}"/>
+    <hyperlink ref="B705" xr:uid="{D13194E0-44A8-554E-B85B-E9CE7EC4F5EF}"/>
+    <hyperlink ref="A708" r:id="rId429" display="https://scholar.google.com/citations?view_op=view_citation&amp;hl=en&amp;user=dq0JfDcAAAAJ&amp;citation_for_view=dq0JfDcAAAAJ:zYLM7Y9cAGgC" xr:uid="{4D8C5D73-9BBD-1247-85F2-B4E8476D31C6}"/>
+    <hyperlink ref="B708" xr:uid="{458D8C43-2E67-DC41-80BE-95C73C272E62}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>